<commit_message>
Testi: didascalie in frase, tour più concreto, ingegnere con un solo saluto
Didascalie di Andamento e Punti deboli in frase invece che a uguali e
puntini; il tour dice cosa fare col file esportato e «Guardali per
primi» al posto di «Un coach parte da qui»; apex anche nel tour;
«dal volante». In inglese l'ingegnere dice sempre «Engineer here».
Il focus generico non ripete più il consiglio del debrief. Il segnaposto
del nome curva è in frase, le gomme dal vivo sono in °C, e il piano di
test (JSON e XLSX) avvia HONE da accoach_main.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HONE_Test_Plan_AC_ACC.xlsx
+++ b/HONE_Test_Plan_AC_ACC.xlsx
@@ -697,7 +697,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Avvio di HONE: doppio click su HONE.bat (oppure launcher / 'python -m accoach ...').</t>
+          <t xml:space="preserve">  • Avvio di HONE: doppio click su HONE.bat (oppure launcher / 'python accoach_main.py ...').</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Avvia AC/ACC ed entra in una sessione di Prova. Avvia HONE (launcher o 'python -m accoach monitor').</t>
+          <t>Avvia AC/ACC ed entra in una sessione di Prova. Avvia HONE (launcher o 'python accoach_main.py monitor').</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">

</xml_diff>